<commit_message>
added products page tests
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/ProductData.xlsx
+++ b/src/test/resources/testdata/ProductData.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Selenium_projects\SauceDemo_Automation\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6074DEF-B5BE-4720-8432-376625268CC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32A90D86-075D-4530-B510-D431BF0F96EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Products" sheetId="1" r:id="rId1"/>
+    <sheet name="Products" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
   <si>
     <t>ProductName</t>
   </si>
@@ -49,6 +49,42 @@
   </si>
   <si>
     <t>Test.allTheThings() T-Shirt (Red)</t>
+  </si>
+  <si>
+    <t>$29.99</t>
+  </si>
+  <si>
+    <t>$9.99</t>
+  </si>
+  <si>
+    <t>$15.99</t>
+  </si>
+  <si>
+    <t>$49.99</t>
+  </si>
+  <si>
+    <t>$7.99</t>
+  </si>
+  <si>
+    <t>ExpectedDescription</t>
+  </si>
+  <si>
+    <t>carry.allTheThings() with the sleek, streamlined Sly Pack that melds uncompromising style with unequaled laptop and tablet protection.</t>
+  </si>
+  <si>
+    <t>Get your testing superhero on with the Sauce Labs bolt T-shirt. From American Apparel, 100% ringspun combed cotton, heather gray with red bolt.</t>
+  </si>
+  <si>
+    <t>A red light isn't the desired state in testing but it sure helps when riding your bike at night. Water-resistant with 3 lighting modes, 1 AAA battery included.</t>
+  </si>
+  <si>
+    <t>It's not every day that you come across a midweight quarter-zip fleece jacket capable of handling everything from a relaxing day outdoors to a busy day at the office.</t>
+  </si>
+  <si>
+    <t>Rib snap infant onesie for the junior automation engineer in development. Reinforced 3-snap bottom closure, two-needle hemmed sleeved and bottom won't unravel.</t>
+  </si>
+  <si>
+    <t>This classic Sauce Labs t-shirt is perfect to wear when cozying up to your keyboard to automate a few tests. Super-soft and comfy ringspun combed cotton.</t>
   </si>
 </sst>
 </file>
@@ -84,8 +120,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -365,68 +407,90 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EAF32E0-844F-4268-BEA7-B8A78E8BA197}">
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.73046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.46484375" customWidth="1"/>
+    <col min="2" max="2" width="19.796875" customWidth="1"/>
+    <col min="3" max="3" width="67.265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A1" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
+      <c r="C1" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2">
-        <v>29.99</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
+      <c r="B2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B3">
-        <v>9.99</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
+      <c r="B3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B4">
-        <v>15.99</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
+      <c r="B4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B5">
-        <v>49.99</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
+      <c r="B5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B6">
-        <v>7.99</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
+      <c r="B6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B7">
-        <v>15.99</v>
+      <c r="B7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>